<commit_message>
perfil-gamer: WILD HEARTS verdict=Bom, drop PS4+PS5 from header, search includes notes, Plano subtracts hours already played on current game
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -3382,7 +3382,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="43" t="inlineStr">
         <is>
@@ -3390,7 +3389,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="18" customHeight="1" s="36">
       <c r="A9" s="44" t="inlineStr">
         <is>
@@ -3668,7 +3666,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="47" t="inlineStr">
         <is>
@@ -3676,7 +3673,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="18" customHeight="1" s="36">
       <c r="A23" s="48" t="inlineStr">
         <is>
@@ -3934,7 +3930,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35" ht="15" customHeight="1" s="36">
       <c r="A35" s="49" t="inlineStr">
         <is>
@@ -3942,7 +3937,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="18" customHeight="1" s="36">
       <c r="A37" s="37" t="inlineStr">
         <is>
@@ -4159,7 +4153,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="36">
       <c r="A48" s="47" t="inlineStr">
         <is>
@@ -4167,7 +4160,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="18" customHeight="1" s="36">
       <c r="A50" s="48" t="inlineStr">
         <is>
@@ -4488,7 +4480,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59"/>
     <row r="60" ht="15" customHeight="1" s="36">
       <c r="A60" s="58" t="inlineStr">
         <is>
@@ -4496,7 +4487,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="18" customHeight="1" s="36">
       <c r="A62" s="59" t="inlineStr">
         <is>
@@ -4605,7 +4595,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="36">
       <c r="A72" s="47" t="inlineStr">
         <is>
@@ -4613,7 +4602,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74" ht="18" customHeight="1" s="36">
       <c r="A74" s="48" t="inlineStr">
         <is>
@@ -5615,6 +5603,11 @@
       <c r="K18" s="62" t="n">
         <v>3</v>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
       <c r="M18" s="68" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="36">

</xml_diff>

<commit_message>
perfil-gamer: WILD HEARTS verdict=Bom, drop PS4+PS5 from header, search includes notes, Plano subtracts hours already played on current game (#46)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -3382,7 +3382,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="43" t="inlineStr">
         <is>
@@ -3390,7 +3389,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="18" customHeight="1" s="36">
       <c r="A9" s="44" t="inlineStr">
         <is>
@@ -3668,7 +3666,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="47" t="inlineStr">
         <is>
@@ -3676,7 +3673,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="18" customHeight="1" s="36">
       <c r="A23" s="48" t="inlineStr">
         <is>
@@ -3934,7 +3930,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35" ht="15" customHeight="1" s="36">
       <c r="A35" s="49" t="inlineStr">
         <is>
@@ -3942,7 +3937,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="18" customHeight="1" s="36">
       <c r="A37" s="37" t="inlineStr">
         <is>
@@ -4159,7 +4153,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="36">
       <c r="A48" s="47" t="inlineStr">
         <is>
@@ -4167,7 +4160,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="18" customHeight="1" s="36">
       <c r="A50" s="48" t="inlineStr">
         <is>
@@ -4488,7 +4480,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59"/>
     <row r="60" ht="15" customHeight="1" s="36">
       <c r="A60" s="58" t="inlineStr">
         <is>
@@ -4496,7 +4487,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="18" customHeight="1" s="36">
       <c r="A62" s="59" t="inlineStr">
         <is>
@@ -4605,7 +4595,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="36">
       <c r="A72" s="47" t="inlineStr">
         <is>
@@ -4613,7 +4602,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74" ht="18" customHeight="1" s="36">
       <c r="A74" s="48" t="inlineStr">
         <is>
@@ -5615,6 +5603,11 @@
       <c r="K18" s="62" t="n">
         <v>3</v>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Bom</t>
+        </is>
+      </c>
       <c r="M18" s="68" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="36">

</xml_diff>

<commit_message>
Add release year field and year filter to Perfil Gamer
Each game now carries an official release year (g.ano), researched from the
web. The Games tab gets a "Ano de lançamento" filter (multi-select chips) and
a "Lançamento" sort option, and the year shows on each card.

- Add Ano (and Grátis) columns to biblioteca_jogos.xlsx; gerar_dados.py reads
  them and emits g.ano in the seed dados.js.
- Cloud is the source of truth, so boot() backfills g.ano on games loaded from
  the cloud by matching the seed by id (name fallback); idempotent.
- Editable in the inline card editor and the "Registrar jogo" modal.
- Bump service worker cache to v6.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017SPZn5KU3cgkRDyUwNpYkx
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -4739,7 +4739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.01171875" defaultRowHeight="14.25" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.03" customWidth="1" style="35" min="1" max="1"/>
@@ -4818,6 +4818,16 @@
           <t>Observação</t>
         </is>
       </c>
+      <c r="N1" s="35" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="O1" s="35" t="inlineStr">
+        <is>
+          <t>Grátis</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1" s="36">
       <c r="A2" s="65" t="n">
@@ -4867,6 +4877,9 @@
         </is>
       </c>
       <c r="M2" s="65" t="n"/>
+      <c r="N2" s="35" t="n">
+        <v>2013</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" s="36">
       <c r="A3" s="68" t="n">
@@ -4915,6 +4928,9 @@
         <is>
           <t>2ª walkthrough: DLCs dos personagens. História/combate medianos mas divertia</t>
         </is>
+      </c>
+      <c r="N3" s="35" t="n">
+        <v>2016</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="36">
@@ -4965,6 +4981,9 @@
           <t>Jogado muito por ser gigante + pandemia, não por qualidade</t>
         </is>
       </c>
+      <c r="N4" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="36">
       <c r="A5" s="68" t="n">
@@ -5010,6 +5029,9 @@
         </is>
       </c>
       <c r="M5" s="65" t="n"/>
+      <c r="N5" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1" s="36">
       <c r="A6" s="65" t="n">
@@ -5055,6 +5077,9 @@
         </is>
       </c>
       <c r="M6" s="68" t="n"/>
+      <c r="N6" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="36">
       <c r="A7" s="68" t="n">
@@ -5102,6 +5127,9 @@
         </is>
       </c>
       <c r="M7" s="65" t="n"/>
+      <c r="N7" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="36">
       <c r="A8" s="65" t="n">
@@ -5147,6 +5175,9 @@
         </is>
       </c>
       <c r="M8" s="68" t="n"/>
+      <c r="N8" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="36">
       <c r="A9" s="68" t="n">
@@ -5194,6 +5225,9 @@
         </is>
       </c>
       <c r="M9" s="65" t="n"/>
+      <c r="N9" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="36">
       <c r="A10" s="65" t="n">
@@ -5239,6 +5273,9 @@
         </is>
       </c>
       <c r="M10" s="68" t="n"/>
+      <c r="N10" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="36">
       <c r="A11" s="68" t="n">
@@ -5284,6 +5321,9 @@
         </is>
       </c>
       <c r="M11" s="65" t="n"/>
+      <c r="N11" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="36">
       <c r="A12" s="65" t="n">
@@ -5333,6 +5373,9 @@
           <t>Inclui Complete Edition (94h PS4) + base (37h PS4) · Nota revisada 1.5→2.5 jul/2026 (161h + zerado + 2 walkthroughs)</t>
         </is>
       </c>
+      <c r="N12" s="35" t="n">
+        <v>2015</v>
+      </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="36">
       <c r="A13" s="68" t="n">
@@ -5378,6 +5421,9 @@
         </is>
       </c>
       <c r="M13" s="65" t="n"/>
+      <c r="N13" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="36">
       <c r="A14" s="65" t="n">
@@ -5423,6 +5469,9 @@
         </is>
       </c>
       <c r="M14" s="68" t="n"/>
+      <c r="N14" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="36">
       <c r="A15" s="68" t="n">
@@ -5468,6 +5517,9 @@
         </is>
       </c>
       <c r="M15" s="65" t="n"/>
+      <c r="N15" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="36">
       <c r="A16" s="65" t="n">
@@ -5513,6 +5565,9 @@
         </is>
       </c>
       <c r="M16" s="68" t="n"/>
+      <c r="N16" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="36">
       <c r="A17" s="68" t="n">
@@ -5560,6 +5615,9 @@
         </is>
       </c>
       <c r="M17" s="65" t="n"/>
+      <c r="N17" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="36">
       <c r="A18" s="65" t="n">
@@ -5603,12 +5661,15 @@
       <c r="K18" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="35" t="inlineStr">
         <is>
           <t>Bom</t>
         </is>
       </c>
       <c r="M18" s="68" t="n"/>
+      <c r="N18" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="36">
       <c r="A19" s="68" t="n">
@@ -5654,6 +5715,9 @@
         </is>
       </c>
       <c r="M19" s="68" t="n"/>
+      <c r="N19" s="35" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="36">
       <c r="A20" s="65" t="n">
@@ -5703,6 +5767,9 @@
         </is>
       </c>
       <c r="M20" s="65" t="n"/>
+      <c r="N20" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="36">
       <c r="A21" s="68" t="n">
@@ -5748,6 +5815,9 @@
         </is>
       </c>
       <c r="M21" s="68" t="n"/>
+      <c r="N21" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="36">
       <c r="A22" s="65" t="n">
@@ -5793,6 +5863,9 @@
         </is>
       </c>
       <c r="M22" s="65" t="n"/>
+      <c r="N22" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="36">
       <c r="A23" s="68" t="n">
@@ -5842,6 +5915,9 @@
           <t>Rezerado jul/2026 (+17h na 2ª walkthrough)</t>
         </is>
       </c>
+      <c r="N23" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="36">
       <c r="A24" s="65" t="n">
@@ -5887,6 +5963,9 @@
         </is>
       </c>
       <c r="M24" s="65" t="n"/>
+      <c r="N24" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="36">
       <c r="A25" s="68" t="n">
@@ -5936,6 +6015,9 @@
           <t>Não gostei do fluxo do jogo, lutas repetidas com os mesmos monstros, genérico</t>
         </is>
       </c>
+      <c r="N25" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="26" ht="16.5" customHeight="1" s="36">
       <c r="A26" s="65" t="n">
@@ -5983,6 +6065,9 @@
         </is>
       </c>
       <c r="M26" s="65" t="n"/>
+      <c r="N26" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="27" ht="16.5" customHeight="1" s="36">
       <c r="A27" s="68" t="n">
@@ -6028,6 +6113,9 @@
         </is>
       </c>
       <c r="M27" s="68" t="n"/>
+      <c r="N27" s="35" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="36">
       <c r="A28" s="65" t="n">
@@ -6077,6 +6165,9 @@
           <t>Jogando no nightmare no ng+ · Comprado por R$60; últimas 4 missões finalizadas jul/2026</t>
         </is>
       </c>
+      <c r="N28" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="29" ht="16.5" customHeight="1" s="36">
       <c r="A29" s="68" t="n">
@@ -6128,6 +6219,9 @@
         </is>
       </c>
       <c r="M29" s="68" t="n"/>
+      <c r="N29" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="30" ht="16.5" customHeight="1" s="36">
       <c r="A30" s="65" t="n">
@@ -6173,6 +6267,9 @@
         </is>
       </c>
       <c r="M30" s="65" t="n"/>
+      <c r="N30" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="31" ht="16.5" customHeight="1" s="36">
       <c r="A31" s="68" t="n">
@@ -6218,6 +6315,9 @@
         </is>
       </c>
       <c r="M31" s="68" t="n"/>
+      <c r="N31" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="32" ht="16.5" customHeight="1" s="36">
       <c r="A32" s="65" t="n">
@@ -6267,6 +6367,9 @@
           <t>Replay jun/2026 (19h): Gameplay 2→3; zerado no fácil para encerrar; sem completar sides. Replay de jogo finalizado, não retentativa.</t>
         </is>
       </c>
+      <c r="N32" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="33" ht="16.5" customHeight="1" s="36">
       <c r="A33" s="68" t="n">
@@ -6314,6 +6417,9 @@
         </is>
       </c>
       <c r="M33" s="65" t="n"/>
+      <c r="N33" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="36">
       <c r="A34" s="65" t="n">
@@ -6359,6 +6465,9 @@
         </is>
       </c>
       <c r="M34" s="68" t="n"/>
+      <c r="N34" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="36">
       <c r="A35" s="68" t="n">
@@ -6408,6 +6517,9 @@
         </is>
       </c>
       <c r="M35" s="65" t="n"/>
+      <c r="N35" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="36">
       <c r="A36" s="65" t="n">
@@ -6455,6 +6567,9 @@
         </is>
       </c>
       <c r="M36" s="65" t="n"/>
+      <c r="N36" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="36">
       <c r="A37" s="68" t="n">
@@ -6500,6 +6615,9 @@
         </is>
       </c>
       <c r="M37" s="65" t="n"/>
+      <c r="N37" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="36">
       <c r="A38" s="65" t="n">
@@ -6549,6 +6667,9 @@
         </is>
       </c>
       <c r="M38" s="68" t="n"/>
+      <c r="N38" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="36">
       <c r="A39" s="68" t="n">
@@ -6598,6 +6719,9 @@
         </is>
       </c>
       <c r="M39" s="65" t="n"/>
+      <c r="N39" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="36">
       <c r="A40" s="65" t="n">
@@ -6643,6 +6767,9 @@
         </is>
       </c>
       <c r="M40" s="68" t="n"/>
+      <c r="N40" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="36">
       <c r="A41" s="68" t="n">
@@ -6690,6 +6817,9 @@
         </is>
       </c>
       <c r="M41" s="65" t="n"/>
+      <c r="N41" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="36">
       <c r="A42" s="65" t="n">
@@ -6739,6 +6869,9 @@
         </is>
       </c>
       <c r="M42" s="68" t="n"/>
+      <c r="N42" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="36">
       <c r="A43" s="68" t="n">
@@ -6786,6 +6919,9 @@
         </is>
       </c>
       <c r="M43" s="65" t="n"/>
+      <c r="N43" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="36">
       <c r="A44" s="65" t="n">
@@ -6833,6 +6969,9 @@
         </is>
       </c>
       <c r="M44" s="68" t="n"/>
+      <c r="N44" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="36">
       <c r="A45" s="68" t="n">
@@ -6878,6 +7017,9 @@
         </is>
       </c>
       <c r="M45" s="65" t="n"/>
+      <c r="N45" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="36">
       <c r="A46" s="65" t="n">
@@ -6927,6 +7069,9 @@
         </is>
       </c>
       <c r="M46" s="68" t="n"/>
+      <c r="N46" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="36">
       <c r="A47" s="68" t="n">
@@ -6972,6 +7117,9 @@
         </is>
       </c>
       <c r="M47" s="65" t="n"/>
+      <c r="N47" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="48" ht="16.5" customHeight="1" s="36">
       <c r="A48" s="65" t="n">
@@ -7021,6 +7169,9 @@
         </is>
       </c>
       <c r="M48" s="68" t="n"/>
+      <c r="N48" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="49" ht="16.5" customHeight="1" s="36">
       <c r="A49" s="68" t="n">
@@ -7070,6 +7221,9 @@
         </is>
       </c>
       <c r="M49" s="65" t="n"/>
+      <c r="N49" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="50" ht="16.5" customHeight="1" s="36">
       <c r="A50" s="65" t="n">
@@ -7115,6 +7269,9 @@
         </is>
       </c>
       <c r="M50" s="68" t="n"/>
+      <c r="N50" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="51" ht="16.5" customHeight="1" s="36">
       <c r="A51" s="68" t="n">
@@ -7164,6 +7321,9 @@
         </is>
       </c>
       <c r="M51" s="65" t="n"/>
+      <c r="N51" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="52" ht="16.5" customHeight="1" s="36">
       <c r="A52" s="65" t="n">
@@ -7213,6 +7373,9 @@
         </is>
       </c>
       <c r="M52" s="68" t="n"/>
+      <c r="N52" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="53" ht="16.5" customHeight="1" s="36">
       <c r="A53" s="68" t="n">
@@ -7262,6 +7425,9 @@
         </is>
       </c>
       <c r="M53" s="65" t="n"/>
+      <c r="N53" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="54" ht="16.5" customHeight="1" s="36">
       <c r="A54" s="65" t="n">
@@ -7315,6 +7481,9 @@
           <t>[Director's Cut PS5] mesma coisa que id 61 é mesmo jogo</t>
         </is>
       </c>
+      <c r="N54" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="55" ht="16.5" customHeight="1" s="36">
       <c r="A55" s="68" t="n">
@@ -7364,6 +7533,12 @@
         </is>
       </c>
       <c r="M55" s="65" t="n"/>
+      <c r="N55" s="35" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O55" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" ht="16.5" customHeight="1" s="36">
       <c r="A56" s="65" t="n">
@@ -7413,6 +7588,9 @@
         </is>
       </c>
       <c r="M56" s="68" t="n"/>
+      <c r="N56" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="57" ht="16.5" customHeight="1" s="36">
       <c r="A57" s="68" t="n">
@@ -7458,6 +7636,9 @@
         </is>
       </c>
       <c r="M57" s="65" t="n"/>
+      <c r="N57" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="58" ht="16.5" customHeight="1" s="36">
       <c r="A58" s="65" t="n">
@@ -7507,6 +7688,9 @@
         </is>
       </c>
       <c r="M58" s="68" t="n"/>
+      <c r="N58" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="59" ht="16.5" customHeight="1" s="36">
       <c r="A59" s="68" t="n">
@@ -7552,6 +7736,9 @@
         </is>
       </c>
       <c r="M59" s="65" t="n"/>
+      <c r="N59" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="60" ht="16.5" customHeight="1" s="36">
       <c r="A60" s="65" t="n">
@@ -7597,6 +7784,9 @@
         </is>
       </c>
       <c r="M60" s="68" t="n"/>
+      <c r="N60" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="61" ht="16.5" customHeight="1" s="36">
       <c r="A61" s="68" t="n">
@@ -7646,6 +7836,9 @@
           <t>Top 3 de todos os tempos; 2 walkthroughs completas</t>
         </is>
       </c>
+      <c r="N61" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="62" ht="16.5" customHeight="1" s="36">
       <c r="A62" s="65" t="n">
@@ -7691,6 +7884,9 @@
         </is>
       </c>
       <c r="M62" s="68" t="n"/>
+      <c r="N62" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="63" ht="16.5" customHeight="1" s="36">
       <c r="A63" s="68" t="n">
@@ -7742,6 +7938,9 @@
         </is>
       </c>
       <c r="M63" s="65" t="n"/>
+      <c r="N63" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="64" ht="16.5" customHeight="1" s="36">
       <c r="A64" s="65" t="n">
@@ -7791,6 +7990,9 @@
         </is>
       </c>
       <c r="M64" s="68" t="n"/>
+      <c r="N64" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="65" ht="16.5" customHeight="1" s="36">
       <c r="A65" s="68" t="n">
@@ -7836,6 +8038,9 @@
         </is>
       </c>
       <c r="M65" s="65" t="n"/>
+      <c r="N65" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="66" ht="16.5" customHeight="1" s="36">
       <c r="A66" s="65" t="n">
@@ -7885,6 +8090,9 @@
         </is>
       </c>
       <c r="M66" s="68" t="n"/>
+      <c r="N66" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="36">
       <c r="A67" s="68" t="n">
@@ -7934,6 +8142,9 @@
         </is>
       </c>
       <c r="M67" s="65" t="n"/>
+      <c r="N67" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="36">
       <c r="A68" s="65" t="n">
@@ -7979,6 +8190,12 @@
         </is>
       </c>
       <c r="M68" s="68" t="n"/>
+      <c r="N68" s="35" t="n">
+        <v>2015</v>
+      </c>
+      <c r="O68" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69" ht="16.5" customHeight="1" s="36">
       <c r="A69" s="68" t="n">
@@ -8024,6 +8241,9 @@
         </is>
       </c>
       <c r="M69" s="65" t="n"/>
+      <c r="N69" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="70" ht="16.5" customHeight="1" s="36">
       <c r="A70" s="68" t="n">
@@ -8069,6 +8289,9 @@
         </is>
       </c>
       <c r="M70" s="65" t="n"/>
+      <c r="N70" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="71" ht="16.5" customHeight="1" s="36">
       <c r="A71" s="65" t="n">
@@ -8118,6 +8341,9 @@
         </is>
       </c>
       <c r="M71" s="68" t="n"/>
+      <c r="N71" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="36">
       <c r="A72" s="65" t="n">
@@ -8171,6 +8397,12 @@
           <t>PS Plus grátis jun/2026. Dropado em ~30 min. Padrão confirmado: souls-like não-FromSoft decepciona.</t>
         </is>
       </c>
+      <c r="N72" s="35" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O72" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73" ht="14.25" customHeight="1" s="36">
       <c r="A73" s="65" t="n">
@@ -8223,6 +8455,9 @@
         <is>
           <t>Jogadas 9h + 4h = 13h total. Dropado jul/2026</t>
         </is>
+      </c>
+      <c r="N73" t="n">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perfil Gamer: ano de lançamento + filtro por ano (#72)
Each game now carries an official release year (g.ano), researched from the
web. The Games tab gets a "Ano de lançamento" filter (multi-select chips) and
a "Lançamento" sort option, and the year shows on each card.

- Add Ano (and Grátis) columns to biblioteca_jogos.xlsx; gerar_dados.py reads
  them and emits g.ano in the seed dados.js.
- Cloud is the source of truth, so boot() backfills g.ano on games loaded from
  the cloud by matching the seed by id (name fallback); idempotent.
- Editable in the inline card editor and the "Registrar jogo" modal.
- Bump service worker cache to v6.


Claude-Session: https://claude.ai/code/session_017SPZn5KU3cgkRDyUwNpYkx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/perfil-gamer-src/biblioteca_jogos.xlsx
+++ b/perfil-gamer-src/biblioteca_jogos.xlsx
@@ -4739,7 +4739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.01171875" defaultRowHeight="14.25" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.03" customWidth="1" style="35" min="1" max="1"/>
@@ -4818,6 +4818,16 @@
           <t>Observação</t>
         </is>
       </c>
+      <c r="N1" s="35" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="O1" s="35" t="inlineStr">
+        <is>
+          <t>Grátis</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1" s="36">
       <c r="A2" s="65" t="n">
@@ -4867,6 +4877,9 @@
         </is>
       </c>
       <c r="M2" s="65" t="n"/>
+      <c r="N2" s="35" t="n">
+        <v>2013</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" s="36">
       <c r="A3" s="68" t="n">
@@ -4915,6 +4928,9 @@
         <is>
           <t>2ª walkthrough: DLCs dos personagens. História/combate medianos mas divertia</t>
         </is>
+      </c>
+      <c r="N3" s="35" t="n">
+        <v>2016</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="36">
@@ -4965,6 +4981,9 @@
           <t>Jogado muito por ser gigante + pandemia, não por qualidade</t>
         </is>
       </c>
+      <c r="N4" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="36">
       <c r="A5" s="68" t="n">
@@ -5010,6 +5029,9 @@
         </is>
       </c>
       <c r="M5" s="65" t="n"/>
+      <c r="N5" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1" s="36">
       <c r="A6" s="65" t="n">
@@ -5055,6 +5077,9 @@
         </is>
       </c>
       <c r="M6" s="68" t="n"/>
+      <c r="N6" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="36">
       <c r="A7" s="68" t="n">
@@ -5102,6 +5127,9 @@
         </is>
       </c>
       <c r="M7" s="65" t="n"/>
+      <c r="N7" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="36">
       <c r="A8" s="65" t="n">
@@ -5147,6 +5175,9 @@
         </is>
       </c>
       <c r="M8" s="68" t="n"/>
+      <c r="N8" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="36">
       <c r="A9" s="68" t="n">
@@ -5194,6 +5225,9 @@
         </is>
       </c>
       <c r="M9" s="65" t="n"/>
+      <c r="N9" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="36">
       <c r="A10" s="65" t="n">
@@ -5239,6 +5273,9 @@
         </is>
       </c>
       <c r="M10" s="68" t="n"/>
+      <c r="N10" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="36">
       <c r="A11" s="68" t="n">
@@ -5284,6 +5321,9 @@
         </is>
       </c>
       <c r="M11" s="65" t="n"/>
+      <c r="N11" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="36">
       <c r="A12" s="65" t="n">
@@ -5333,6 +5373,9 @@
           <t>Inclui Complete Edition (94h PS4) + base (37h PS4) · Nota revisada 1.5→2.5 jul/2026 (161h + zerado + 2 walkthroughs)</t>
         </is>
       </c>
+      <c r="N12" s="35" t="n">
+        <v>2015</v>
+      </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="36">
       <c r="A13" s="68" t="n">
@@ -5378,6 +5421,9 @@
         </is>
       </c>
       <c r="M13" s="65" t="n"/>
+      <c r="N13" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="36">
       <c r="A14" s="65" t="n">
@@ -5423,6 +5469,9 @@
         </is>
       </c>
       <c r="M14" s="68" t="n"/>
+      <c r="N14" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="36">
       <c r="A15" s="68" t="n">
@@ -5468,6 +5517,9 @@
         </is>
       </c>
       <c r="M15" s="65" t="n"/>
+      <c r="N15" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="36">
       <c r="A16" s="65" t="n">
@@ -5513,6 +5565,9 @@
         </is>
       </c>
       <c r="M16" s="68" t="n"/>
+      <c r="N16" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="36">
       <c r="A17" s="68" t="n">
@@ -5560,6 +5615,9 @@
         </is>
       </c>
       <c r="M17" s="65" t="n"/>
+      <c r="N17" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="36">
       <c r="A18" s="65" t="n">
@@ -5603,12 +5661,15 @@
       <c r="K18" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="35" t="inlineStr">
         <is>
           <t>Bom</t>
         </is>
       </c>
       <c r="M18" s="68" t="n"/>
+      <c r="N18" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="36">
       <c r="A19" s="68" t="n">
@@ -5654,6 +5715,9 @@
         </is>
       </c>
       <c r="M19" s="68" t="n"/>
+      <c r="N19" s="35" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="36">
       <c r="A20" s="65" t="n">
@@ -5703,6 +5767,9 @@
         </is>
       </c>
       <c r="M20" s="65" t="n"/>
+      <c r="N20" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="36">
       <c r="A21" s="68" t="n">
@@ -5748,6 +5815,9 @@
         </is>
       </c>
       <c r="M21" s="68" t="n"/>
+      <c r="N21" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="36">
       <c r="A22" s="65" t="n">
@@ -5793,6 +5863,9 @@
         </is>
       </c>
       <c r="M22" s="65" t="n"/>
+      <c r="N22" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="36">
       <c r="A23" s="68" t="n">
@@ -5842,6 +5915,9 @@
           <t>Rezerado jul/2026 (+17h na 2ª walkthrough)</t>
         </is>
       </c>
+      <c r="N23" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="36">
       <c r="A24" s="65" t="n">
@@ -5887,6 +5963,9 @@
         </is>
       </c>
       <c r="M24" s="65" t="n"/>
+      <c r="N24" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="36">
       <c r="A25" s="68" t="n">
@@ -5936,6 +6015,9 @@
           <t>Não gostei do fluxo do jogo, lutas repetidas com os mesmos monstros, genérico</t>
         </is>
       </c>
+      <c r="N25" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="26" ht="16.5" customHeight="1" s="36">
       <c r="A26" s="65" t="n">
@@ -5983,6 +6065,9 @@
         </is>
       </c>
       <c r="M26" s="65" t="n"/>
+      <c r="N26" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="27" ht="16.5" customHeight="1" s="36">
       <c r="A27" s="68" t="n">
@@ -6028,6 +6113,9 @@
         </is>
       </c>
       <c r="M27" s="68" t="n"/>
+      <c r="N27" s="35" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="36">
       <c r="A28" s="65" t="n">
@@ -6077,6 +6165,9 @@
           <t>Jogando no nightmare no ng+ · Comprado por R$60; últimas 4 missões finalizadas jul/2026</t>
         </is>
       </c>
+      <c r="N28" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="29" ht="16.5" customHeight="1" s="36">
       <c r="A29" s="68" t="n">
@@ -6128,6 +6219,9 @@
         </is>
       </c>
       <c r="M29" s="68" t="n"/>
+      <c r="N29" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="30" ht="16.5" customHeight="1" s="36">
       <c r="A30" s="65" t="n">
@@ -6173,6 +6267,9 @@
         </is>
       </c>
       <c r="M30" s="65" t="n"/>
+      <c r="N30" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="31" ht="16.5" customHeight="1" s="36">
       <c r="A31" s="68" t="n">
@@ -6218,6 +6315,9 @@
         </is>
       </c>
       <c r="M31" s="68" t="n"/>
+      <c r="N31" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="32" ht="16.5" customHeight="1" s="36">
       <c r="A32" s="65" t="n">
@@ -6267,6 +6367,9 @@
           <t>Replay jun/2026 (19h): Gameplay 2→3; zerado no fácil para encerrar; sem completar sides. Replay de jogo finalizado, não retentativa.</t>
         </is>
       </c>
+      <c r="N32" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="33" ht="16.5" customHeight="1" s="36">
       <c r="A33" s="68" t="n">
@@ -6314,6 +6417,9 @@
         </is>
       </c>
       <c r="M33" s="65" t="n"/>
+      <c r="N33" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="36">
       <c r="A34" s="65" t="n">
@@ -6359,6 +6465,9 @@
         </is>
       </c>
       <c r="M34" s="68" t="n"/>
+      <c r="N34" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="36">
       <c r="A35" s="68" t="n">
@@ -6408,6 +6517,9 @@
         </is>
       </c>
       <c r="M35" s="65" t="n"/>
+      <c r="N35" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="36">
       <c r="A36" s="65" t="n">
@@ -6455,6 +6567,9 @@
         </is>
       </c>
       <c r="M36" s="65" t="n"/>
+      <c r="N36" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="36">
       <c r="A37" s="68" t="n">
@@ -6500,6 +6615,9 @@
         </is>
       </c>
       <c r="M37" s="65" t="n"/>
+      <c r="N37" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="36">
       <c r="A38" s="65" t="n">
@@ -6549,6 +6667,9 @@
         </is>
       </c>
       <c r="M38" s="68" t="n"/>
+      <c r="N38" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="36">
       <c r="A39" s="68" t="n">
@@ -6598,6 +6719,9 @@
         </is>
       </c>
       <c r="M39" s="65" t="n"/>
+      <c r="N39" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="36">
       <c r="A40" s="65" t="n">
@@ -6643,6 +6767,9 @@
         </is>
       </c>
       <c r="M40" s="68" t="n"/>
+      <c r="N40" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="36">
       <c r="A41" s="68" t="n">
@@ -6690,6 +6817,9 @@
         </is>
       </c>
       <c r="M41" s="65" t="n"/>
+      <c r="N41" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="36">
       <c r="A42" s="65" t="n">
@@ -6739,6 +6869,9 @@
         </is>
       </c>
       <c r="M42" s="68" t="n"/>
+      <c r="N42" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="36">
       <c r="A43" s="68" t="n">
@@ -6786,6 +6919,9 @@
         </is>
       </c>
       <c r="M43" s="65" t="n"/>
+      <c r="N43" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="36">
       <c r="A44" s="65" t="n">
@@ -6833,6 +6969,9 @@
         </is>
       </c>
       <c r="M44" s="68" t="n"/>
+      <c r="N44" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="36">
       <c r="A45" s="68" t="n">
@@ -6878,6 +7017,9 @@
         </is>
       </c>
       <c r="M45" s="65" t="n"/>
+      <c r="N45" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="36">
       <c r="A46" s="65" t="n">
@@ -6927,6 +7069,9 @@
         </is>
       </c>
       <c r="M46" s="68" t="n"/>
+      <c r="N46" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="36">
       <c r="A47" s="68" t="n">
@@ -6972,6 +7117,9 @@
         </is>
       </c>
       <c r="M47" s="65" t="n"/>
+      <c r="N47" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="48" ht="16.5" customHeight="1" s="36">
       <c r="A48" s="65" t="n">
@@ -7021,6 +7169,9 @@
         </is>
       </c>
       <c r="M48" s="68" t="n"/>
+      <c r="N48" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="49" ht="16.5" customHeight="1" s="36">
       <c r="A49" s="68" t="n">
@@ -7070,6 +7221,9 @@
         </is>
       </c>
       <c r="M49" s="65" t="n"/>
+      <c r="N49" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="50" ht="16.5" customHeight="1" s="36">
       <c r="A50" s="65" t="n">
@@ -7115,6 +7269,9 @@
         </is>
       </c>
       <c r="M50" s="68" t="n"/>
+      <c r="N50" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="51" ht="16.5" customHeight="1" s="36">
       <c r="A51" s="68" t="n">
@@ -7164,6 +7321,9 @@
         </is>
       </c>
       <c r="M51" s="65" t="n"/>
+      <c r="N51" s="35" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="52" ht="16.5" customHeight="1" s="36">
       <c r="A52" s="65" t="n">
@@ -7213,6 +7373,9 @@
         </is>
       </c>
       <c r="M52" s="68" t="n"/>
+      <c r="N52" s="35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="53" ht="16.5" customHeight="1" s="36">
       <c r="A53" s="68" t="n">
@@ -7262,6 +7425,9 @@
         </is>
       </c>
       <c r="M53" s="65" t="n"/>
+      <c r="N53" s="35" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="54" ht="16.5" customHeight="1" s="36">
       <c r="A54" s="65" t="n">
@@ -7315,6 +7481,9 @@
           <t>[Director's Cut PS5] mesma coisa que id 61 é mesmo jogo</t>
         </is>
       </c>
+      <c r="N54" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="55" ht="16.5" customHeight="1" s="36">
       <c r="A55" s="68" t="n">
@@ -7364,6 +7533,12 @@
         </is>
       </c>
       <c r="M55" s="65" t="n"/>
+      <c r="N55" s="35" t="n">
+        <v>2024</v>
+      </c>
+      <c r="O55" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" ht="16.5" customHeight="1" s="36">
       <c r="A56" s="65" t="n">
@@ -7413,6 +7588,9 @@
         </is>
       </c>
       <c r="M56" s="68" t="n"/>
+      <c r="N56" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="57" ht="16.5" customHeight="1" s="36">
       <c r="A57" s="68" t="n">
@@ -7458,6 +7636,9 @@
         </is>
       </c>
       <c r="M57" s="65" t="n"/>
+      <c r="N57" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="58" ht="16.5" customHeight="1" s="36">
       <c r="A58" s="65" t="n">
@@ -7507,6 +7688,9 @@
         </is>
       </c>
       <c r="M58" s="68" t="n"/>
+      <c r="N58" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="59" ht="16.5" customHeight="1" s="36">
       <c r="A59" s="68" t="n">
@@ -7552,6 +7736,9 @@
         </is>
       </c>
       <c r="M59" s="65" t="n"/>
+      <c r="N59" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="60" ht="16.5" customHeight="1" s="36">
       <c r="A60" s="65" t="n">
@@ -7597,6 +7784,9 @@
         </is>
       </c>
       <c r="M60" s="68" t="n"/>
+      <c r="N60" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="61" ht="16.5" customHeight="1" s="36">
       <c r="A61" s="68" t="n">
@@ -7646,6 +7836,9 @@
           <t>Top 3 de todos os tempos; 2 walkthroughs completas</t>
         </is>
       </c>
+      <c r="N61" s="35" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="62" ht="16.5" customHeight="1" s="36">
       <c r="A62" s="65" t="n">
@@ -7691,6 +7884,9 @@
         </is>
       </c>
       <c r="M62" s="68" t="n"/>
+      <c r="N62" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="63" ht="16.5" customHeight="1" s="36">
       <c r="A63" s="68" t="n">
@@ -7742,6 +7938,9 @@
         </is>
       </c>
       <c r="M63" s="65" t="n"/>
+      <c r="N63" s="35" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="64" ht="16.5" customHeight="1" s="36">
       <c r="A64" s="65" t="n">
@@ -7791,6 +7990,9 @@
         </is>
       </c>
       <c r="M64" s="68" t="n"/>
+      <c r="N64" s="35" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="65" ht="16.5" customHeight="1" s="36">
       <c r="A65" s="68" t="n">
@@ -7836,6 +8038,9 @@
         </is>
       </c>
       <c r="M65" s="65" t="n"/>
+      <c r="N65" s="35" t="n">
+        <v>2026</v>
+      </c>
     </row>
     <row r="66" ht="16.5" customHeight="1" s="36">
       <c r="A66" s="65" t="n">
@@ -7885,6 +8090,9 @@
         </is>
       </c>
       <c r="M66" s="68" t="n"/>
+      <c r="N66" s="35" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="36">
       <c r="A67" s="68" t="n">
@@ -7934,6 +8142,9 @@
         </is>
       </c>
       <c r="M67" s="65" t="n"/>
+      <c r="N67" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="36">
       <c r="A68" s="65" t="n">
@@ -7979,6 +8190,12 @@
         </is>
       </c>
       <c r="M68" s="68" t="n"/>
+      <c r="N68" s="35" t="n">
+        <v>2015</v>
+      </c>
+      <c r="O68" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="69" ht="16.5" customHeight="1" s="36">
       <c r="A69" s="68" t="n">
@@ -8024,6 +8241,9 @@
         </is>
       </c>
       <c r="M69" s="65" t="n"/>
+      <c r="N69" s="35" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="70" ht="16.5" customHeight="1" s="36">
       <c r="A70" s="68" t="n">
@@ -8069,6 +8289,9 @@
         </is>
       </c>
       <c r="M70" s="65" t="n"/>
+      <c r="N70" s="35" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="71" ht="16.5" customHeight="1" s="36">
       <c r="A71" s="65" t="n">
@@ -8118,6 +8341,9 @@
         </is>
       </c>
       <c r="M71" s="68" t="n"/>
+      <c r="N71" s="35" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="36">
       <c r="A72" s="65" t="n">
@@ -8171,6 +8397,12 @@
           <t>PS Plus grátis jun/2026. Dropado em ~30 min. Padrão confirmado: souls-like não-FromSoft decepciona.</t>
         </is>
       </c>
+      <c r="N72" s="35" t="n">
+        <v>2025</v>
+      </c>
+      <c r="O72" s="35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="73" ht="14.25" customHeight="1" s="36">
       <c r="A73" s="65" t="n">
@@ -8223,6 +8455,9 @@
         <is>
           <t>Jogadas 9h + 4h = 13h total. Dropado jul/2026</t>
         </is>
+      </c>
+      <c r="N73" t="n">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>